<commit_message>
Add AWS public rate refresh for cost workbook
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -615,70 +615,82 @@
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2. Main inputs</t>
+          <t>Refresh AWS public rates</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Select the AWS region and enter data volume, object count, wave size, archive mix, restore tier, retention and FastConnect/Direct Connect assumptions.</t>
+          <t>Run: python3 tools/refresh_cost_calculator_rates.py --regions sa-east-1,us-east-1. It calls the same public Amazon S3 and AWS Data Transfer catalog endpoints used by Raijin. It updates AWS public rate columns only; FastConnect/Direct Connect, Deep Archive storage and OCI fields remain under customer control.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>3. AWS estimate</t>
+          <t>2. Main inputs</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Shows charged AWS-side components. Outbound is optional and can use a specific FastConnect/Direct Connect rate when entered.</t>
+          <t>Select the AWS region and enter data volume, object count, wave size, archive mix, restore tier, retention and FastConnect/Direct Connect assumptions.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>4. OCI estimate</t>
+          <t>3. AWS estimate</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Separates one-time write requests, storage accrued while data arrives, and the recurring final Object Storage cost.</t>
+          <t>Shows charged AWS-side components. Outbound is optional and can use a specific FastConnect/Direct Connect rate when entered.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>5. Early delete</t>
+          <t>4. OCI estimate</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Add one or more groups of Deep Archive objects by volume and average archive age. The model calculates the 180-day minimum-storage remainder.</t>
+          <t>Separates one-time write requests, storage accrued while data arrives, and the recurring final Object Storage cost.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. Summary</t>
+          <t>5. Early delete</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Use this tab for the executive view. It intentionally keeps recurring OCI storage separate from one-time migration costs.</t>
+          <t>Add one or more groups of Deep Archive objects by volume and average archive age. The model calculates the 180-day minimum-storage remainder.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>6. Summary</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Use this tab for the executive view. It intentionally keeps recurring OCI storage separate from one-time migration costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>All TB/GB inputs use decimal units (1 TB = 1,000 GB), matching cloud price-list units. Taxes, credits, enterprise discounts, source-storage charges, VM cost and partner circuit charges are excluded unless you add them manually.</t>
         </is>

</xml_diff>

<commit_message>
Focus cost calculator on public AWS internet pricing
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tariffs by region'!$A$4:$O$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tariffs by region'!$A$4:$L$54</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -711,7 +711,7 @@
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Include AWS outbound</t>
+          <t>Preserve S3 tags</t>
         </is>
       </c>
       <c r="B14" s="5" t="b">
@@ -719,112 +719,35 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Turn off only if outbound is intentionally excluded.</t>
+          <t>Adds one S3 GET/TAG request per file.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Outbound tariff</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>FastConnect</t>
-        </is>
+          <t>Early Deep Archive delete data (TB)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Public AWS or FastConnect/Direct Connect tariff from the regional table.</t>
+          <t>Volume deleted after migration; leave zero when data stays in S3.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="29" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Include OCI storage</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="b">
-        <v>1</v>
+          <t>Average Deep Archive age (days)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>180</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Includes OCI write requests, accrued storage and final recurring storage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="29" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Estimated migration duration (days)</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>47</v>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Used only to estimate OCI storage accumulated while data arrives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="29" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>OCI write operations per file</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>1 for small files; increase for multipart uploads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="29" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Preserve S3 tags</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Adds one S3 GET/TAG request per file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="29" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Early Deep Archive delete data (TB)</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Volume deleted after migration; leave zero when data stays in S3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="29" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Average Deep Archive age (days)</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="n">
-        <v>180</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>AWS charges the remaining portion of the 180-day commitment.</t>
         </is>
@@ -847,15 +770,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="B14 B16 B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"BULK,STANDARD"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Public AWS,FastConnect"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -868,24 +788,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="46" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="58" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -898,7 +815,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Enter public or contractual values. The refresh script updates the AWS public columns for sa-east-1/us-east-1; circuit, Deep Archive storage and OCI values remain your inputs.</t>
+          <t>Use only public AWS list prices. The refresh script updates supported AWS public columns for sa-east-1/us-east-1.</t>
         </is>
       </c>
     </row>
@@ -915,79 +832,61 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>AWS outbound
+          <t>AWS Internet outbound
 USD/GB</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>FastConnect / Direct Connect
-outbound USD/GB</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Deep Archive storage
 USD/GB-month</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Deep Archive BULK retrieval
 USD/GB</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Deep Archive STANDARD retrieval
 USD/GB</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Temporary S3 Standard restore
 USD/GB-month</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>S3 PUT/LIST
 USD/1,000</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>S3 GET/TAG
 USD/1,000</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Batch job
 USD/job</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Batch object
 USD/1,000</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>OCI Standard storage
-USD/GB-month</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>OCI writes
-USD/10,000</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Notes / source</t>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Public source / notes</t>
         </is>
       </c>
     </row>
@@ -1006,37 +905,30 @@
         <v>0.15</v>
       </c>
       <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
+      <c r="E5" s="10" t="n">
+        <v>0.008</v>
+      </c>
       <c r="F5" s="10" t="n">
-        <v>0.008</v>
+        <v>0.028</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.028</v>
+        <v>0.0405</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>0.0405</v>
+        <v>0.007</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>0.007</v>
+        <v>0.00056</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.00056</v>
+        <v>0.25</v>
       </c>
       <c r="K5" s="10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L5" s="10" t="n">
         <v>1.5e-05</v>
       </c>
-      <c r="M5" s="10" t="n">
-        <v>0.0255</v>
-      </c>
-      <c r="N5" s="10" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>AWS public values collected by Raijin on 2026-08-19; validate contracted rates before approval.</t>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>AWS public values collected by Raijin on 2026-08-19. Refresh before approving spend.</t>
         </is>
       </c>
     </row>
@@ -1055,37 +947,30 @@
         <v>0.09</v>
       </c>
       <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
+      <c r="E6" s="10" t="n">
+        <v>0.0025</v>
+      </c>
       <c r="F6" s="10" t="n">
-        <v>0.0025</v>
+        <v>0.02</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.02</v>
+        <v>0.0125</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>0.0125</v>
+        <v>0.055</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>0.055</v>
+        <v>0.0004</v>
       </c>
       <c r="J6" s="10" t="n">
-        <v>0.0004</v>
+        <v>0.25</v>
       </c>
       <c r="K6" s="10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L6" s="10" t="n">
         <v>0.001</v>
       </c>
-      <c r="M6" s="10" t="n">
-        <v>0.0255</v>
-      </c>
-      <c r="N6" s="10" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Example values; use the refresh script or contractual values.</t>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Example public values; refresh before use.</t>
         </is>
       </c>
     </row>
@@ -1101,10 +986,7 @@
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="10" t="n"/>
       <c r="K7" s="10" t="n"/>
-      <c r="L7" s="10" t="n"/>
-      <c r="M7" s="10" t="n"/>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
@@ -1118,10 +1000,7 @@
       <c r="I8" s="10" t="n"/>
       <c r="J8" s="10" t="n"/>
       <c r="K8" s="10" t="n"/>
-      <c r="L8" s="10" t="n"/>
-      <c r="M8" s="10" t="n"/>
-      <c r="N8" s="10" t="n"/>
-      <c r="O8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -1135,10 +1014,7 @@
       <c r="I9" s="10" t="n"/>
       <c r="J9" s="10" t="n"/>
       <c r="K9" s="10" t="n"/>
-      <c r="L9" s="10" t="n"/>
-      <c r="M9" s="10" t="n"/>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
@@ -1152,10 +1028,7 @@
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="10" t="n"/>
       <c r="K10" s="10" t="n"/>
-      <c r="L10" s="10" t="n"/>
-      <c r="M10" s="10" t="n"/>
-      <c r="N10" s="10" t="n"/>
-      <c r="O10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -1169,10 +1042,7 @@
       <c r="I11" s="10" t="n"/>
       <c r="J11" s="10" t="n"/>
       <c r="K11" s="10" t="n"/>
-      <c r="L11" s="10" t="n"/>
-      <c r="M11" s="10" t="n"/>
-      <c r="N11" s="10" t="n"/>
-      <c r="O11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
@@ -1186,10 +1056,7 @@
       <c r="I12" s="10" t="n"/>
       <c r="J12" s="10" t="n"/>
       <c r="K12" s="10" t="n"/>
-      <c r="L12" s="10" t="n"/>
-      <c r="M12" s="10" t="n"/>
-      <c r="N12" s="10" t="n"/>
-      <c r="O12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -1203,10 +1070,7 @@
       <c r="I13" s="10" t="n"/>
       <c r="J13" s="10" t="n"/>
       <c r="K13" s="10" t="n"/>
-      <c r="L13" s="10" t="n"/>
-      <c r="M13" s="10" t="n"/>
-      <c r="N13" s="10" t="n"/>
-      <c r="O13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
@@ -1220,10 +1084,7 @@
       <c r="I14" s="10" t="n"/>
       <c r="J14" s="10" t="n"/>
       <c r="K14" s="10" t="n"/>
-      <c r="L14" s="10" t="n"/>
-      <c r="M14" s="10" t="n"/>
-      <c r="N14" s="10" t="n"/>
-      <c r="O14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -1237,10 +1098,7 @@
       <c r="I15" s="10" t="n"/>
       <c r="J15" s="10" t="n"/>
       <c r="K15" s="10" t="n"/>
-      <c r="L15" s="10" t="n"/>
-      <c r="M15" s="10" t="n"/>
-      <c r="N15" s="10" t="n"/>
-      <c r="O15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
@@ -1254,10 +1112,7 @@
       <c r="I16" s="10" t="n"/>
       <c r="J16" s="10" t="n"/>
       <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="n"/>
-      <c r="M16" s="10" t="n"/>
-      <c r="N16" s="10" t="n"/>
-      <c r="O16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1271,10 +1126,7 @@
       <c r="I17" s="10" t="n"/>
       <c r="J17" s="10" t="n"/>
       <c r="K17" s="10" t="n"/>
-      <c r="L17" s="10" t="n"/>
-      <c r="M17" s="10" t="n"/>
-      <c r="N17" s="10" t="n"/>
-      <c r="O17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
@@ -1288,10 +1140,7 @@
       <c r="I18" s="10" t="n"/>
       <c r="J18" s="10" t="n"/>
       <c r="K18" s="10" t="n"/>
-      <c r="L18" s="10" t="n"/>
-      <c r="M18" s="10" t="n"/>
-      <c r="N18" s="10" t="n"/>
-      <c r="O18" s="5" t="n"/>
+      <c r="L18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1305,10 +1154,7 @@
       <c r="I19" s="10" t="n"/>
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="10" t="n"/>
-      <c r="L19" s="10" t="n"/>
-      <c r="M19" s="10" t="n"/>
-      <c r="N19" s="10" t="n"/>
-      <c r="O19" s="5" t="n"/>
+      <c r="L19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
@@ -1322,10 +1168,7 @@
       <c r="I20" s="10" t="n"/>
       <c r="J20" s="10" t="n"/>
       <c r="K20" s="10" t="n"/>
-      <c r="L20" s="10" t="n"/>
-      <c r="M20" s="10" t="n"/>
-      <c r="N20" s="10" t="n"/>
-      <c r="O20" s="5" t="n"/>
+      <c r="L20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1339,10 +1182,7 @@
       <c r="I21" s="10" t="n"/>
       <c r="J21" s="10" t="n"/>
       <c r="K21" s="10" t="n"/>
-      <c r="L21" s="10" t="n"/>
-      <c r="M21" s="10" t="n"/>
-      <c r="N21" s="10" t="n"/>
-      <c r="O21" s="5" t="n"/>
+      <c r="L21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1356,10 +1196,7 @@
       <c r="I22" s="10" t="n"/>
       <c r="J22" s="10" t="n"/>
       <c r="K22" s="10" t="n"/>
-      <c r="L22" s="10" t="n"/>
-      <c r="M22" s="10" t="n"/>
-      <c r="N22" s="10" t="n"/>
-      <c r="O22" s="5" t="n"/>
+      <c r="L22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1373,10 +1210,7 @@
       <c r="I23" s="10" t="n"/>
       <c r="J23" s="10" t="n"/>
       <c r="K23" s="10" t="n"/>
-      <c r="L23" s="10" t="n"/>
-      <c r="M23" s="10" t="n"/>
-      <c r="N23" s="10" t="n"/>
-      <c r="O23" s="5" t="n"/>
+      <c r="L23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
@@ -1390,10 +1224,7 @@
       <c r="I24" s="10" t="n"/>
       <c r="J24" s="10" t="n"/>
       <c r="K24" s="10" t="n"/>
-      <c r="L24" s="10" t="n"/>
-      <c r="M24" s="10" t="n"/>
-      <c r="N24" s="10" t="n"/>
-      <c r="O24" s="5" t="n"/>
+      <c r="L24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1407,10 +1238,7 @@
       <c r="I25" s="10" t="n"/>
       <c r="J25" s="10" t="n"/>
       <c r="K25" s="10" t="n"/>
-      <c r="L25" s="10" t="n"/>
-      <c r="M25" s="10" t="n"/>
-      <c r="N25" s="10" t="n"/>
-      <c r="O25" s="5" t="n"/>
+      <c r="L25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
@@ -1424,10 +1252,7 @@
       <c r="I26" s="10" t="n"/>
       <c r="J26" s="10" t="n"/>
       <c r="K26" s="10" t="n"/>
-      <c r="L26" s="10" t="n"/>
-      <c r="M26" s="10" t="n"/>
-      <c r="N26" s="10" t="n"/>
-      <c r="O26" s="5" t="n"/>
+      <c r="L26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1441,10 +1266,7 @@
       <c r="I27" s="10" t="n"/>
       <c r="J27" s="10" t="n"/>
       <c r="K27" s="10" t="n"/>
-      <c r="L27" s="10" t="n"/>
-      <c r="M27" s="10" t="n"/>
-      <c r="N27" s="10" t="n"/>
-      <c r="O27" s="5" t="n"/>
+      <c r="L27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
@@ -1458,10 +1280,7 @@
       <c r="I28" s="10" t="n"/>
       <c r="J28" s="10" t="n"/>
       <c r="K28" s="10" t="n"/>
-      <c r="L28" s="10" t="n"/>
-      <c r="M28" s="10" t="n"/>
-      <c r="N28" s="10" t="n"/>
-      <c r="O28" s="5" t="n"/>
+      <c r="L28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1475,10 +1294,7 @@
       <c r="I29" s="10" t="n"/>
       <c r="J29" s="10" t="n"/>
       <c r="K29" s="10" t="n"/>
-      <c r="L29" s="10" t="n"/>
-      <c r="M29" s="10" t="n"/>
-      <c r="N29" s="10" t="n"/>
-      <c r="O29" s="5" t="n"/>
+      <c r="L29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
@@ -1492,10 +1308,7 @@
       <c r="I30" s="10" t="n"/>
       <c r="J30" s="10" t="n"/>
       <c r="K30" s="10" t="n"/>
-      <c r="L30" s="10" t="n"/>
-      <c r="M30" s="10" t="n"/>
-      <c r="N30" s="10" t="n"/>
-      <c r="O30" s="5" t="n"/>
+      <c r="L30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1509,10 +1322,7 @@
       <c r="I31" s="10" t="n"/>
       <c r="J31" s="10" t="n"/>
       <c r="K31" s="10" t="n"/>
-      <c r="L31" s="10" t="n"/>
-      <c r="M31" s="10" t="n"/>
-      <c r="N31" s="10" t="n"/>
-      <c r="O31" s="5" t="n"/>
+      <c r="L31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
@@ -1526,10 +1336,7 @@
       <c r="I32" s="10" t="n"/>
       <c r="J32" s="10" t="n"/>
       <c r="K32" s="10" t="n"/>
-      <c r="L32" s="10" t="n"/>
-      <c r="M32" s="10" t="n"/>
-      <c r="N32" s="10" t="n"/>
-      <c r="O32" s="5" t="n"/>
+      <c r="L32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1543,10 +1350,7 @@
       <c r="I33" s="10" t="n"/>
       <c r="J33" s="10" t="n"/>
       <c r="K33" s="10" t="n"/>
-      <c r="L33" s="10" t="n"/>
-      <c r="M33" s="10" t="n"/>
-      <c r="N33" s="10" t="n"/>
-      <c r="O33" s="5" t="n"/>
+      <c r="L33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n"/>
@@ -1560,10 +1364,7 @@
       <c r="I34" s="10" t="n"/>
       <c r="J34" s="10" t="n"/>
       <c r="K34" s="10" t="n"/>
-      <c r="L34" s="10" t="n"/>
-      <c r="M34" s="10" t="n"/>
-      <c r="N34" s="10" t="n"/>
-      <c r="O34" s="5" t="n"/>
+      <c r="L34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1577,10 +1378,7 @@
       <c r="I35" s="10" t="n"/>
       <c r="J35" s="10" t="n"/>
       <c r="K35" s="10" t="n"/>
-      <c r="L35" s="10" t="n"/>
-      <c r="M35" s="10" t="n"/>
-      <c r="N35" s="10" t="n"/>
-      <c r="O35" s="5" t="n"/>
+      <c r="L35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n"/>
@@ -1594,10 +1392,7 @@
       <c r="I36" s="10" t="n"/>
       <c r="J36" s="10" t="n"/>
       <c r="K36" s="10" t="n"/>
-      <c r="L36" s="10" t="n"/>
-      <c r="M36" s="10" t="n"/>
-      <c r="N36" s="10" t="n"/>
-      <c r="O36" s="5" t="n"/>
+      <c r="L36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1611,10 +1406,7 @@
       <c r="I37" s="10" t="n"/>
       <c r="J37" s="10" t="n"/>
       <c r="K37" s="10" t="n"/>
-      <c r="L37" s="10" t="n"/>
-      <c r="M37" s="10" t="n"/>
-      <c r="N37" s="10" t="n"/>
-      <c r="O37" s="5" t="n"/>
+      <c r="L37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n"/>
@@ -1628,10 +1420,7 @@
       <c r="I38" s="10" t="n"/>
       <c r="J38" s="10" t="n"/>
       <c r="K38" s="10" t="n"/>
-      <c r="L38" s="10" t="n"/>
-      <c r="M38" s="10" t="n"/>
-      <c r="N38" s="10" t="n"/>
-      <c r="O38" s="5" t="n"/>
+      <c r="L38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1645,10 +1434,7 @@
       <c r="I39" s="10" t="n"/>
       <c r="J39" s="10" t="n"/>
       <c r="K39" s="10" t="n"/>
-      <c r="L39" s="10" t="n"/>
-      <c r="M39" s="10" t="n"/>
-      <c r="N39" s="10" t="n"/>
-      <c r="O39" s="5" t="n"/>
+      <c r="L39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n"/>
@@ -1662,10 +1448,7 @@
       <c r="I40" s="10" t="n"/>
       <c r="J40" s="10" t="n"/>
       <c r="K40" s="10" t="n"/>
-      <c r="L40" s="10" t="n"/>
-      <c r="M40" s="10" t="n"/>
-      <c r="N40" s="10" t="n"/>
-      <c r="O40" s="5" t="n"/>
+      <c r="L40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1679,10 +1462,7 @@
       <c r="I41" s="10" t="n"/>
       <c r="J41" s="10" t="n"/>
       <c r="K41" s="10" t="n"/>
-      <c r="L41" s="10" t="n"/>
-      <c r="M41" s="10" t="n"/>
-      <c r="N41" s="10" t="n"/>
-      <c r="O41" s="5" t="n"/>
+      <c r="L41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -1696,10 +1476,7 @@
       <c r="I42" s="10" t="n"/>
       <c r="J42" s="10" t="n"/>
       <c r="K42" s="10" t="n"/>
-      <c r="L42" s="10" t="n"/>
-      <c r="M42" s="10" t="n"/>
-      <c r="N42" s="10" t="n"/>
-      <c r="O42" s="5" t="n"/>
+      <c r="L42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1713,10 +1490,7 @@
       <c r="I43" s="10" t="n"/>
       <c r="J43" s="10" t="n"/>
       <c r="K43" s="10" t="n"/>
-      <c r="L43" s="10" t="n"/>
-      <c r="M43" s="10" t="n"/>
-      <c r="N43" s="10" t="n"/>
-      <c r="O43" s="5" t="n"/>
+      <c r="L43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n"/>
@@ -1730,10 +1504,7 @@
       <c r="I44" s="10" t="n"/>
       <c r="J44" s="10" t="n"/>
       <c r="K44" s="10" t="n"/>
-      <c r="L44" s="10" t="n"/>
-      <c r="M44" s="10" t="n"/>
-      <c r="N44" s="10" t="n"/>
-      <c r="O44" s="5" t="n"/>
+      <c r="L44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1747,10 +1518,7 @@
       <c r="I45" s="10" t="n"/>
       <c r="J45" s="10" t="n"/>
       <c r="K45" s="10" t="n"/>
-      <c r="L45" s="10" t="n"/>
-      <c r="M45" s="10" t="n"/>
-      <c r="N45" s="10" t="n"/>
-      <c r="O45" s="5" t="n"/>
+      <c r="L45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n"/>
@@ -1764,10 +1532,7 @@
       <c r="I46" s="10" t="n"/>
       <c r="J46" s="10" t="n"/>
       <c r="K46" s="10" t="n"/>
-      <c r="L46" s="10" t="n"/>
-      <c r="M46" s="10" t="n"/>
-      <c r="N46" s="10" t="n"/>
-      <c r="O46" s="5" t="n"/>
+      <c r="L46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1781,10 +1546,7 @@
       <c r="I47" s="10" t="n"/>
       <c r="J47" s="10" t="n"/>
       <c r="K47" s="10" t="n"/>
-      <c r="L47" s="10" t="n"/>
-      <c r="M47" s="10" t="n"/>
-      <c r="N47" s="10" t="n"/>
-      <c r="O47" s="5" t="n"/>
+      <c r="L47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -1798,10 +1560,7 @@
       <c r="I48" s="10" t="n"/>
       <c r="J48" s="10" t="n"/>
       <c r="K48" s="10" t="n"/>
-      <c r="L48" s="10" t="n"/>
-      <c r="M48" s="10" t="n"/>
-      <c r="N48" s="10" t="n"/>
-      <c r="O48" s="5" t="n"/>
+      <c r="L48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1815,10 +1574,7 @@
       <c r="I49" s="10" t="n"/>
       <c r="J49" s="10" t="n"/>
       <c r="K49" s="10" t="n"/>
-      <c r="L49" s="10" t="n"/>
-      <c r="M49" s="10" t="n"/>
-      <c r="N49" s="10" t="n"/>
-      <c r="O49" s="5" t="n"/>
+      <c r="L49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n"/>
@@ -1832,10 +1588,7 @@
       <c r="I50" s="10" t="n"/>
       <c r="J50" s="10" t="n"/>
       <c r="K50" s="10" t="n"/>
-      <c r="L50" s="10" t="n"/>
-      <c r="M50" s="10" t="n"/>
-      <c r="N50" s="10" t="n"/>
-      <c r="O50" s="5" t="n"/>
+      <c r="L50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1849,10 +1602,7 @@
       <c r="I51" s="10" t="n"/>
       <c r="J51" s="10" t="n"/>
       <c r="K51" s="10" t="n"/>
-      <c r="L51" s="10" t="n"/>
-      <c r="M51" s="10" t="n"/>
-      <c r="N51" s="10" t="n"/>
-      <c r="O51" s="5" t="n"/>
+      <c r="L51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n"/>
@@ -1866,10 +1616,7 @@
       <c r="I52" s="10" t="n"/>
       <c r="J52" s="10" t="n"/>
       <c r="K52" s="10" t="n"/>
-      <c r="L52" s="10" t="n"/>
-      <c r="M52" s="10" t="n"/>
-      <c r="N52" s="10" t="n"/>
-      <c r="O52" s="5" t="n"/>
+      <c r="L52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1883,10 +1630,7 @@
       <c r="I53" s="10" t="n"/>
       <c r="J53" s="10" t="n"/>
       <c r="K53" s="10" t="n"/>
-      <c r="L53" s="10" t="n"/>
-      <c r="M53" s="10" t="n"/>
-      <c r="N53" s="10" t="n"/>
-      <c r="O53" s="5" t="n"/>
+      <c r="L53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n"/>
@@ -1900,16 +1644,13 @@
       <c r="I54" s="10" t="n"/>
       <c r="J54" s="10" t="n"/>
       <c r="K54" s="10" t="n"/>
-      <c r="L54" s="10" t="n"/>
-      <c r="M54" s="10" t="n"/>
-      <c r="N54" s="10" t="n"/>
-      <c r="O54" s="5" t="n"/>
+      <c r="L54" s="5" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O54"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1921,7 +1662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -1930,20 +1671,21 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Migration cost summary</t>
+          <t>AWS migration cost summary</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The one-time project cost excludes the recurring OCI monthly storage cost, shown separately at the bottom.</t>
+          <t>All values are AWS public-price estimates. Set the checkbox beside outbound to FALSE to exclude it from all totals.</t>
         </is>
       </c>
     </row>
@@ -1983,6 +1725,11 @@
           <t>Calculation / note</t>
         </is>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Include outbound?</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -2000,12 +1747,12 @@
         </is>
       </c>
       <c r="D5" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,6,FALSE)</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,5,FALSE)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F5" s="12">
@@ -2017,6 +1764,11 @@
           <t>Only the Deep Archive share.</t>
         </is>
       </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -2034,12 +1786,12 @@
         </is>
       </c>
       <c r="D6" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,7,FALSE)</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,6,FALSE)</f>
         <v/>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F6" s="12">
@@ -2051,6 +1803,11 @@
           <t>Only the Deep Archive share.</t>
         </is>
       </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2068,12 +1825,12 @@
         </is>
       </c>
       <c r="D7" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,8,FALSE)</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,7,FALSE)</f>
         <v/>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F7" s="12">
@@ -2085,6 +1842,11 @@
           <t>Temporary S3 Standard copy after restore.</t>
         </is>
       </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -2102,12 +1864,12 @@
         </is>
       </c>
       <c r="D8" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,11,FALSE)</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,10,FALSE)</f>
         <v/>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F8" s="12">
@@ -2119,6 +1881,11 @@
           <t>One restore job per archive wave.</t>
         </is>
       </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -2136,12 +1903,12 @@
         </is>
       </c>
       <c r="D9" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,12,FALSE)/1000</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,11,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F9" s="12">
@@ -2153,6 +1920,11 @@
           <t>Object-task rate normalized to one object.</t>
         </is>
       </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -2170,12 +1942,12 @@
         </is>
       </c>
       <c r="D10" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,9,FALSE)/1000</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,8,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F10" s="12">
@@ -2187,6 +1959,11 @@
           <t>Conservative ListObjectsV2 estimate.</t>
         </is>
       </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -2204,12 +1981,12 @@
         </is>
       </c>
       <c r="D11" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,10,FALSE)/1000</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,9,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F11" s="12">
@@ -2221,6 +1998,11 @@
           <t>One streaming GetObject per object.</t>
         </is>
       </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -2238,28 +2020,33 @@
         </is>
       </c>
       <c r="D12" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,10,FALSE)/1000</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,9,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F12" s="12">
-        <f>IF('Transfer data'!B19,IFERROR(B12*D12,"Not priced"),0)</f>
+        <f>IF('Transfer data'!B14,IFERROR(B12*D12,"Not priced"),0)</f>
         <v/>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Only when tag preservation is enabled.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>AWS outbound to OCI</t>
+          <t>AWS outbound</t>
         </is>
       </c>
       <c r="B13" s="11">
@@ -2272,22 +2059,25 @@
         </is>
       </c>
       <c r="D13" s="12">
-        <f>IF('Transfer data'!B15="FastConnect",IFERROR(IF(VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,4,FALSE)&gt;0,VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,4,FALSE),VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,3,FALSE)),VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,3,FALSE)),VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,3,FALSE))</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,3,FALSE)</f>
         <v/>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Selected outbound tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F13" s="12">
-        <f>IF('Transfer data'!B14,IFERROR(B13*D13,"Not priced"),0)</f>
+        <f>IF(H13,IFERROR(B13*D13,"Not priced"),0)</f>
         <v/>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>FastConnect falls back to public AWS when its rate is blank.</t>
-        </is>
+          <t>Use the checkbox to include or exclude outbound.</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2297,7 +2087,7 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>'Transfer data'!B20*1000*MAX(0,180-'Transfer data'!B21)/30</f>
+        <f>'Transfer data'!B15*1000*MAX(0,180-'Transfer data'!B16)/30</f>
         <v/>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -2306,16 +2096,16 @@
         </is>
       </c>
       <c r="D14" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,5,FALSE)</f>
+        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,4,FALSE)</f>
         <v/>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>AWS tariff</t>
+          <t>Public AWS</t>
         </is>
       </c>
       <c r="F14" s="12">
-        <f>IF('Transfer data'!B20&gt;0,IFERROR(B14*D14,"Not priced"),0)</f>
+        <f>IF('Transfer data'!B15&gt;0,IFERROR(B14*D14,"Not priced"),0)</f>
         <v/>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -2323,159 +2113,56 @@
           <t>Whole-project early-delete estimate.</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>OCI write requests</t>
-        </is>
-      </c>
-      <c r="B15" s="11">
-        <f>ROUNDUP('Transfer data'!B7/'Transfer data'!B9,0)*'Transfer data'!B18</f>
-        <v/>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>operations / wave</t>
-        </is>
-      </c>
-      <c r="D15" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,14,FALSE)/10000</f>
-        <v/>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>OCI tariff</t>
-        </is>
-      </c>
-      <c r="F15" s="12">
-        <f>IF('Transfer data'!B16,IFERROR(B15*D15,"Not priced"),0)</f>
-        <v/>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Set operations/file to 1 for small files; increase for multipart.</t>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>OCI storage during migration</t>
-        </is>
-      </c>
-      <c r="B16" s="11">
-        <f>'Transfer data'!B6*1000*'Transfer data'!B17/2/30</f>
-        <v/>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>GB-month / project</t>
-        </is>
-      </c>
-      <c r="D16" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,13,FALSE)</f>
-        <v/>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>OCI tariff</t>
-        </is>
-      </c>
-      <c r="F16" s="12">
-        <f>IF('Transfer data'!B16,IFERROR(B16*D16,"Not priced"),0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Linear-arrival approximation over migration duration.</t>
-        </is>
-      </c>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>One-time cost / wave</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="14">
+        <f>SUM(F5:F13)</f>
+        <v/>
+      </c>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>OCI final storage</t>
-        </is>
-      </c>
-      <c r="B17" s="11">
-        <f>'Transfer data'!B6*1000</f>
-        <v/>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>GB-month / project</t>
-        </is>
-      </c>
-      <c r="D17" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:O,13,FALSE)</f>
-        <v/>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>OCI tariff</t>
-        </is>
-      </c>
-      <c r="F17" s="12">
-        <f>IF('Transfer data'!B16,IFERROR(B17*D17,"Not priced"),0)</f>
-        <v/>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Recurring monthly destination cost; excluded from one-time total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>One-time cost / wave</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="14">
-        <f>SUM(F5:F13)+F15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>One-time cost / project</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="14">
-        <f>F20*'Transfer data'!B9+F14+F16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>OCI recurring final cost / month</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="14">
-        <f>F17</f>
-        <v/>
-      </c>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="14">
+        <f>F16*'Transfer data'!B9+F14</f>
+        <v/>
+      </c>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Translate AWS cost calculator workbook
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Transfer data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tariffs by region" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dados da transferência" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tarifas por região" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tariffs by region'!$A$4:$L$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tarifas por região'!$A$4:$L$54</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -540,38 +540,38 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RAIJIN — Transfer data</t>
+          <t>RAIJIN — Dados da transferência</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edit only yellow cells. Use decimal units: 1 TB = 1,000 GB. Costs are calculated in the Summary sheet.</t>
+          <t>Preencha somente as células amarelas. Use unidades decimais: 1 TB = 1.000 GB. Os custos são calculados automaticamente na aba Resumo.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Informação</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Valor</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>O que informar e impacto no cálculo</t>
         </is>
       </c>
     </row>
     <row r="5" ht="29" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>AWS region</t>
+          <t>Região AWS</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -581,14 +581,14 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Select a region listed in ‘Tariffs by region’.</t>
+          <t>Informe o código da região do bucket de origem, por exemplo sa-east-1 ou us-east-1. Deve existir uma linha correspondente na aba Tarifas por região.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="29" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Total data to transfer (TB)</t>
+          <t>Dados totais a transferir (TB)</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -596,14 +596,14 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Total source data, in decimal TB.</t>
+          <t>Informe todo o volume da origem em TB decimais. Exemplo: 600 significa 600.000 GB. É usado no custo total e na quantidade de waves.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="29" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Total files</t>
+          <t>Quantidade total de arquivos</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -611,14 +611,14 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Number of objects discovered in S3.</t>
+          <t>Informe a quantidade de objetos do discovery S3. Ela determina as estimativas de requests, Batch Operations e polling.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="29" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Wave size (TB)</t>
+          <t>Tamanho máximo da wave (TB)</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -626,14 +626,14 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Maximum payload per wave.</t>
+          <t>Informe o limite de dados por wave. A planilha arredonda a quantidade de waves para cima; a última pode ser menor.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="29" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Calculated waves</t>
+          <t>Quantidade calculada de waves</t>
         </is>
       </c>
       <c r="B9" s="8">
@@ -642,14 +642,14 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Calculated automatically.</t>
+          <t>Campo calculado automaticamente a partir dos dados totais e do tamanho máximo da wave. Não editar.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="29" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Deep Archive share</t>
+          <t>Percentual em Deep Archive</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
@@ -657,14 +657,14 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>1 = all data is Deep Archive; 0.5 = half the data.</t>
+          <t>Informe uma fração entre 0 e 1. Use 1 para 100% dos dados em DEEP_ARCHIVE, 0,5 para 50%. Apenas essa parcela recebe custos de restore.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="29" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Restore tier</t>
+          <t>Tier de restore</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -674,14 +674,14 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>BULK or STANDARD.</t>
+          <t>Selecione BULK para menor custo e maior prazo, ou STANDARD para maior velocidade e custo. Aplica-se à parcela Deep Archive.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="29" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Restore retention (days)</t>
+          <t>Retenção do restore (dias)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -689,14 +689,14 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Temporary S3 Standard copy retention after restore is available.</t>
+          <t>Informe por quantos dias a cópia temporária S3 Standard ficará disponível após o restore terminar. Para Deep Archive BULK, 2 dias é a opção mais segura.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="29" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Expected polling cycles per wave</t>
+          <t>Ciclos esperados de polling por wave</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -704,14 +704,14 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Used for the conservative polling request estimate.</t>
+          <t>Informe quantas verificações de disponibilidade a plataforma deve fazer, em média, até o restore ficar pronto. É uma estimativa conservadora de requests.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Preserve S3 tags</t>
+          <t>Preservar tags S3</t>
         </is>
       </c>
       <c r="B14" s="5" t="b">
@@ -719,14 +719,14 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Adds one S3 GET/TAG request per file.</t>
+          <t>Use TRUE quando as tags S3 devem ser copiadas. Isso adiciona uma leitura GET/TAG por arquivo. Use FALSE quando tags não são necessárias.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Early Deep Archive delete data (TB)</t>
+          <t>Dados Deep Archive a excluir antecipadamente (TB)</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
@@ -734,14 +734,14 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Volume deleted after migration; leave zero when data stays in S3.</t>
+          <t>Informe apenas o volume que será excluído ou movido de Deep Archive antes de completar 180 dias. Use zero se os dados permanecerem no S3.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="29" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Average Deep Archive age (days)</t>
+          <t>Idade média no Deep Archive (dias)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
@@ -749,7 +749,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>AWS charges the remaining portion of the 180-day commitment.</t>
+          <t>Informe a idade média ponderada desde a entrada no Deep Archive — não use LastModified se a transição foi por lifecycle. Com 180 ou mais, não há cobrança antecipada.</t>
         </is>
       </c>
     </row>
@@ -808,85 +808,85 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tariffs by region</t>
+          <t>Tarifas por região</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Use only public AWS list prices. The refresh script updates supported AWS public columns for sa-east-1/us-east-1.</t>
+          <t>Use somente preços públicos AWS. O script de atualização preenche as colunas públicas suportadas para sa-east-1 e us-east-1.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>AWS region</t>
+          <t>Região AWS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>Moeda</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>AWS Internet outbound
-USD/GB</t>
+          <t>Outbound AWS Internet
+US$/GB</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Deep Archive storage
-USD/GB-month</t>
+          <t>Armazenamento Deep Archive
+US$/GB-mês</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Deep Archive BULK retrieval
-USD/GB</t>
+          <t>Recuperação Deep Archive BULK
+US$/GB</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Deep Archive STANDARD retrieval
-USD/GB</t>
+          <t>Recuperação Deep Archive STANDARD
+US$/GB</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Temporary S3 Standard restore
-USD/GB-month</t>
+          <t>Cópia temporária S3 Standard
+US$/GB-mês</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>S3 PUT/LIST
-USD/1,000</t>
+US$/1.000</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>S3 GET/TAG
-USD/1,000</t>
+US$/1.000</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Batch job
-USD/job</t>
+          <t>Job Batch
+US$/job</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Batch object
-USD/1,000</t>
+          <t>Objeto Batch
+US$/1.000</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Public source / notes</t>
+          <t>Fonte pública / observações</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>AWS public values collected by Raijin on 2026-08-19. Refresh before approving spend.</t>
+          <t>Valores públicos AWS coletados pelo Raijin em 19/08/2026. Atualize antes de aprovar gastos.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Example public values; refresh before use.</t>
+          <t>Valores públicos de exemplo. Atualize antes de usar.</t>
         </is>
       </c>
     </row>
@@ -1678,90 +1678,90 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AWS migration cost summary</t>
+          <t>Resumo de custo da migração AWS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All values are AWS public-price estimates. Set the checkbox beside outbound to FALSE to exclude it from all totals.</t>
+          <t>Todos os valores são estimativas com preços públicos AWS. Altere a chave ao lado de outbound para FALSE para excluí-lo dos totais.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Métrica</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>Quantidade</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Unidade</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Rate used</t>
+          <t>Tarifa usada</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Rate source</t>
+          <t>Fonte da tarifa</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Estimated cost</t>
+          <t>Custo estimado</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Calculation / note</t>
+          <t>Cálculo / observação</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Include outbound?</t>
+          <t>Incluir outbound?</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Deep Archive BULK retrieval</t>
+          <t>Recuperação Deep Archive BULK</t>
         </is>
       </c>
       <c r="B5" s="11">
-        <f>'Transfer data'!B8*1000*'Transfer data'!B10</f>
+        <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10</f>
         <v/>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>GB / wave</t>
+          <t>GB / onda</t>
         </is>
       </c>
       <c r="D5" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,5,FALSE)</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,5,FALSE)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F5" s="12">
-        <f>IF('Transfer data'!B11="BULK",IFERROR(B5*D5,"Not priced"),0)</f>
+        <f>IF('Dados da transferência'!B11="BULK",IFERROR(B5*D5,"Não precificado"),0)</f>
         <v/>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Only the Deep Archive share.</t>
+          <t>Somente a parcela em Deep Archive.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1773,34 +1773,34 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Deep Archive STANDARD retrieval</t>
+          <t>Recuperação Deep Archive STANDARD</t>
         </is>
       </c>
       <c r="B6" s="11">
-        <f>'Transfer data'!B8*1000*'Transfer data'!B10</f>
+        <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10</f>
         <v/>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>GB / wave</t>
+          <t>GB / onda</t>
         </is>
       </c>
       <c r="D6" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,6,FALSE)</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,6,FALSE)</f>
         <v/>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F6" s="12">
-        <f>IF('Transfer data'!B11="STANDARD",IFERROR(B6*D6,"Not priced"),0)</f>
+        <f>IF('Dados da transferência'!B11="STANDARD",IFERROR(B6*D6,"Não precificado"),0)</f>
         <v/>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Only the Deep Archive share.</t>
+          <t>Somente a parcela em Deep Archive.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -1812,34 +1812,34 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Temporary restored copy</t>
+          <t>Cópia temporária restaurada</t>
         </is>
       </c>
       <c r="B7" s="11">
-        <f>'Transfer data'!B8*1000*'Transfer data'!B10*'Transfer data'!B12/30</f>
+        <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10*'Dados da transferência'!B12/30</f>
         <v/>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>GB-month / wave</t>
+          <t>GB-mês / onda</t>
         </is>
       </c>
       <c r="D7" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,7,FALSE)</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,7,FALSE)</f>
         <v/>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F7" s="12">
-        <f>IFERROR(B7*D7,"Not priced")</f>
+        <f>IFERROR(B7*D7,"Não precificado")</f>
         <v/>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Temporary S3 Standard copy after restore.</t>
+          <t>Cópia S3 Standard temporária após o restore.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1860,25 +1860,25 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>job / wave</t>
+          <t>job / onda</t>
         </is>
       </c>
       <c r="D8" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,10,FALSE)</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,10,FALSE)</f>
         <v/>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F8" s="12">
-        <f>IFERROR(B8*D8,"Not priced")</f>
+        <f>IFERROR(B8*D8,"Não precificado")</f>
         <v/>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>One restore job per archive wave.</t>
+          <t>Um job de restore por onda arquivada.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1890,34 +1890,34 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>S3 Batch object tasks</t>
+          <t>Tarefas de objeto S3 Batch</t>
         </is>
       </c>
       <c r="B9" s="11">
-        <f>ROUNDUP('Transfer data'!B7/'Transfer data'!B9,0)</f>
+        <f>ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9,0)</f>
         <v/>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>objects / wave</t>
+          <t>objetos / onda</t>
         </is>
       </c>
       <c r="D9" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,11,FALSE)/1000</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,11,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F9" s="12">
-        <f>IFERROR(B9*D9,"Not priced")</f>
+        <f>IFERROR(B9*D9,"Não precificado")</f>
         <v/>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Object-task rate normalized to one object.</t>
+          <t>Tarifa de objeto normalizada para uma unidade.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1929,34 +1929,34 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Discovery + restore polling</t>
+          <t>Discovery e polling de restore</t>
         </is>
       </c>
       <c r="B10" s="11">
-        <f>(ROUNDUP('Transfer data'!B7/1000,0)*'Transfer data'!B13)+ROUNDUP('Transfer data'!B7/'Transfer data'!B9/1000,0)</f>
+        <f>(ROUNDUP('Dados da transferência'!B7/1000,0)*'Dados da transferência'!B13)+ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9/1000,0)</f>
         <v/>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>requests / wave</t>
+          <t>solicitações / onda</t>
         </is>
       </c>
       <c r="D10" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,8,FALSE)/1000</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,8,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F10" s="12">
-        <f>IFERROR(B10*D10,"Not priced")</f>
+        <f>IFERROR(B10*D10,"Não precificado")</f>
         <v/>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Conservative ListObjectsV2 estimate.</t>
+          <t>Estimativa conservadora baseada em ListObjectsV2.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1968,34 +1968,34 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>S3 object reads</t>
+          <t>Leituras de objetos S3</t>
         </is>
       </c>
       <c r="B11" s="11">
-        <f>ROUNDUP('Transfer data'!B7/'Transfer data'!B9,0)</f>
+        <f>ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9,0)</f>
         <v/>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>requests / wave</t>
+          <t>solicitações / onda</t>
         </is>
       </c>
       <c r="D11" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,9,FALSE)/1000</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,9,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F11" s="12">
-        <f>IFERROR(B11*D11,"Not priced")</f>
+        <f>IFERROR(B11*D11,"Não precificado")</f>
         <v/>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>One streaming GetObject per object.</t>
+          <t>Um GetObject em streaming por arquivo.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -2007,34 +2007,34 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>S3 tag reads</t>
+          <t>Leituras de tags S3</t>
         </is>
       </c>
       <c r="B12" s="11">
-        <f>ROUNDUP('Transfer data'!B7/'Transfer data'!B9,0)</f>
+        <f>ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9,0)</f>
         <v/>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>requests / wave</t>
+          <t>solicitações / onda</t>
         </is>
       </c>
       <c r="D12" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,9,FALSE)/1000</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,9,FALSE)/1000</f>
         <v/>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F12" s="12">
-        <f>IF('Transfer data'!B14,IFERROR(B12*D12,"Not priced"),0)</f>
+        <f>IF('Dados da transferência'!B14,IFERROR(B12*D12,"Não precificado"),0)</f>
         <v/>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Only when tag preservation is enabled.</t>
+          <t>Somente se a preservação de tags estiver habilitada.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -2046,34 +2046,34 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>AWS outbound</t>
+          <t>Outbound AWS</t>
         </is>
       </c>
       <c r="B13" s="11">
-        <f>'Transfer data'!B8*1000</f>
+        <f>'Dados da transferência'!B8*1000</f>
         <v/>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>GB / wave</t>
+          <t>GB / onda</t>
         </is>
       </c>
       <c r="D13" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,3,FALSE)</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,3,FALSE)</f>
         <v/>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F13" s="12">
-        <f>IF(H13,IFERROR(B13*D13,"Not priced"),0)</f>
+        <f>IF(H13,IFERROR(B13*D13,"Não precificado"),0)</f>
         <v/>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Use the checkbox to include or exclude outbound.</t>
+          <t>Use a chave para incluir ou excluir outbound.</t>
         </is>
       </c>
       <c r="H13" s="5" t="b">
@@ -2083,34 +2083,34 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Early Deep Archive deletion</t>
+          <t>Exclusão antecipada Deep Archive</t>
         </is>
       </c>
       <c r="B14" s="11">
-        <f>'Transfer data'!B15*1000*MAX(0,180-'Transfer data'!B16)/30</f>
+        <f>'Dados da transferência'!B15*1000*MAX(0,180-'Dados da transferência'!B16)/30</f>
         <v/>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>GB-month / project</t>
+          <t>GB-mês / projeto</t>
         </is>
       </c>
       <c r="D14" s="12">
-        <f>VLOOKUP('Transfer data'!B5,'Tariffs by region'!A:L,4,FALSE)</f>
+        <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:L,4,FALSE)</f>
         <v/>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Public AWS</t>
+          <t>AWS pública</t>
         </is>
       </c>
       <c r="F14" s="12">
-        <f>IF('Transfer data'!B15&gt;0,IFERROR(B14*D14,"Not priced"),0)</f>
+        <f>IF('Dados da transferência'!B15&gt;0,IFERROR(B14*D14,"Não precificado"),0)</f>
         <v/>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Whole-project early-delete estimate.</t>
+          <t>Estimativa da exclusão antecipada para todo o projeto.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -2122,7 +2122,7 @@
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>One-time cost / wave</t>
+          <t>Custo único por wave</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
@@ -2139,7 +2139,7 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>One-time cost / project</t>
+          <t>Custo único do projeto</t>
         </is>
       </c>
       <c r="B17" s="4" t="n"/>
@@ -2147,7 +2147,7 @@
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="14">
-        <f>F16*'Transfer data'!B9+F14</f>
+        <f>F16*'Dados da transferência'!B9+F14</f>
         <v/>
       </c>
       <c r="G17" s="4" t="n"/>

</xml_diff>

<commit_message>
Format cost calculator monetary values
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -20,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.00;[Red]-#,##0.00;—"/>
     <numFmt numFmtId="165" formatCode="#,##0.;[Red]-#,##0.;—"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="US$ #,##0.00;[Red]-US$ #,##0.00;—"/>
+    <numFmt numFmtId="167" formatCode="$ #,##0.000000;[Red]-$ #,##0.000000;$ 0.000000"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000;[Red]-#,##0.0000;—"/>
+    <numFmt numFmtId="169" formatCode="$ #,##0.00;[Red]-$ #,##0.00;$ 0.00"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -90,7 +91,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00166534"/>
+        <fgColor rgb="000F5132"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -158,10 +159,13 @@
     <xf numFmtId="167" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -890,7 +894,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="27" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>sa-east-1</t>
@@ -932,7 +936,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="27" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
           <t>us-east-1</t>
@@ -974,7 +978,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="5" t="n"/>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="10" t="n"/>
@@ -988,7 +992,7 @@
       <c r="K7" s="10" t="n"/>
       <c r="L7" s="5" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="5" t="n"/>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="10" t="n"/>
@@ -1002,7 +1006,7 @@
       <c r="K8" s="10" t="n"/>
       <c r="L8" s="5" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="5" t="n"/>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="10" t="n"/>
@@ -1016,7 +1020,7 @@
       <c r="K9" s="10" t="n"/>
       <c r="L9" s="5" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="5" t="n"/>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="10" t="n"/>
@@ -1030,7 +1034,7 @@
       <c r="K10" s="10" t="n"/>
       <c r="L10" s="5" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="5" t="n"/>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="10" t="n"/>
@@ -1044,7 +1048,7 @@
       <c r="K11" s="10" t="n"/>
       <c r="L11" s="5" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="5" t="n"/>
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="10" t="n"/>
@@ -1058,7 +1062,7 @@
       <c r="K12" s="10" t="n"/>
       <c r="L12" s="5" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="5" t="n"/>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="10" t="n"/>
@@ -1072,7 +1076,7 @@
       <c r="K13" s="10" t="n"/>
       <c r="L13" s="5" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="5" t="n"/>
       <c r="B14" s="5" t="n"/>
       <c r="C14" s="10" t="n"/>
@@ -1086,7 +1090,7 @@
       <c r="K14" s="10" t="n"/>
       <c r="L14" s="5" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="27" customHeight="1">
       <c r="A15" s="5" t="n"/>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="10" t="n"/>
@@ -1100,7 +1104,7 @@
       <c r="K15" s="10" t="n"/>
       <c r="L15" s="5" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="27" customHeight="1">
       <c r="A16" s="5" t="n"/>
       <c r="B16" s="5" t="n"/>
       <c r="C16" s="10" t="n"/>
@@ -1114,7 +1118,7 @@
       <c r="K16" s="10" t="n"/>
       <c r="L16" s="5" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="27" customHeight="1">
       <c r="A17" s="5" t="n"/>
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="10" t="n"/>
@@ -1128,7 +1132,7 @@
       <c r="K17" s="10" t="n"/>
       <c r="L17" s="5" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="27" customHeight="1">
       <c r="A18" s="5" t="n"/>
       <c r="B18" s="5" t="n"/>
       <c r="C18" s="10" t="n"/>
@@ -1142,7 +1146,7 @@
       <c r="K18" s="10" t="n"/>
       <c r="L18" s="5" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="27" customHeight="1">
       <c r="A19" s="5" t="n"/>
       <c r="B19" s="5" t="n"/>
       <c r="C19" s="10" t="n"/>
@@ -1156,7 +1160,7 @@
       <c r="K19" s="10" t="n"/>
       <c r="L19" s="5" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="27" customHeight="1">
       <c r="A20" s="5" t="n"/>
       <c r="B20" s="5" t="n"/>
       <c r="C20" s="10" t="n"/>
@@ -1170,7 +1174,7 @@
       <c r="K20" s="10" t="n"/>
       <c r="L20" s="5" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="27" customHeight="1">
       <c r="A21" s="5" t="n"/>
       <c r="B21" s="5" t="n"/>
       <c r="C21" s="10" t="n"/>
@@ -1184,7 +1188,7 @@
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="5" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="27" customHeight="1">
       <c r="A22" s="5" t="n"/>
       <c r="B22" s="5" t="n"/>
       <c r="C22" s="10" t="n"/>
@@ -1198,7 +1202,7 @@
       <c r="K22" s="10" t="n"/>
       <c r="L22" s="5" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="27" customHeight="1">
       <c r="A23" s="5" t="n"/>
       <c r="B23" s="5" t="n"/>
       <c r="C23" s="10" t="n"/>
@@ -1212,7 +1216,7 @@
       <c r="K23" s="10" t="n"/>
       <c r="L23" s="5" t="n"/>
     </row>
-    <row r="24">
+    <row r="24" ht="27" customHeight="1">
       <c r="A24" s="5" t="n"/>
       <c r="B24" s="5" t="n"/>
       <c r="C24" s="10" t="n"/>
@@ -1226,7 +1230,7 @@
       <c r="K24" s="10" t="n"/>
       <c r="L24" s="5" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="27" customHeight="1">
       <c r="A25" s="5" t="n"/>
       <c r="B25" s="5" t="n"/>
       <c r="C25" s="10" t="n"/>
@@ -1240,7 +1244,7 @@
       <c r="K25" s="10" t="n"/>
       <c r="L25" s="5" t="n"/>
     </row>
-    <row r="26">
+    <row r="26" ht="27" customHeight="1">
       <c r="A26" s="5" t="n"/>
       <c r="B26" s="5" t="n"/>
       <c r="C26" s="10" t="n"/>
@@ -1254,7 +1258,7 @@
       <c r="K26" s="10" t="n"/>
       <c r="L26" s="5" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="27" customHeight="1">
       <c r="A27" s="5" t="n"/>
       <c r="B27" s="5" t="n"/>
       <c r="C27" s="10" t="n"/>
@@ -1268,7 +1272,7 @@
       <c r="K27" s="10" t="n"/>
       <c r="L27" s="5" t="n"/>
     </row>
-    <row r="28">
+    <row r="28" ht="27" customHeight="1">
       <c r="A28" s="5" t="n"/>
       <c r="B28" s="5" t="n"/>
       <c r="C28" s="10" t="n"/>
@@ -1282,7 +1286,7 @@
       <c r="K28" s="10" t="n"/>
       <c r="L28" s="5" t="n"/>
     </row>
-    <row r="29">
+    <row r="29" ht="27" customHeight="1">
       <c r="A29" s="5" t="n"/>
       <c r="B29" s="5" t="n"/>
       <c r="C29" s="10" t="n"/>
@@ -1296,7 +1300,7 @@
       <c r="K29" s="10" t="n"/>
       <c r="L29" s="5" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" ht="27" customHeight="1">
       <c r="A30" s="5" t="n"/>
       <c r="B30" s="5" t="n"/>
       <c r="C30" s="10" t="n"/>
@@ -1310,7 +1314,7 @@
       <c r="K30" s="10" t="n"/>
       <c r="L30" s="5" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" ht="27" customHeight="1">
       <c r="A31" s="5" t="n"/>
       <c r="B31" s="5" t="n"/>
       <c r="C31" s="10" t="n"/>
@@ -1324,7 +1328,7 @@
       <c r="K31" s="10" t="n"/>
       <c r="L31" s="5" t="n"/>
     </row>
-    <row r="32">
+    <row r="32" ht="27" customHeight="1">
       <c r="A32" s="5" t="n"/>
       <c r="B32" s="5" t="n"/>
       <c r="C32" s="10" t="n"/>
@@ -1338,7 +1342,7 @@
       <c r="K32" s="10" t="n"/>
       <c r="L32" s="5" t="n"/>
     </row>
-    <row r="33">
+    <row r="33" ht="27" customHeight="1">
       <c r="A33" s="5" t="n"/>
       <c r="B33" s="5" t="n"/>
       <c r="C33" s="10" t="n"/>
@@ -1352,7 +1356,7 @@
       <c r="K33" s="10" t="n"/>
       <c r="L33" s="5" t="n"/>
     </row>
-    <row r="34">
+    <row r="34" ht="27" customHeight="1">
       <c r="A34" s="5" t="n"/>
       <c r="B34" s="5" t="n"/>
       <c r="C34" s="10" t="n"/>
@@ -1366,7 +1370,7 @@
       <c r="K34" s="10" t="n"/>
       <c r="L34" s="5" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" ht="27" customHeight="1">
       <c r="A35" s="5" t="n"/>
       <c r="B35" s="5" t="n"/>
       <c r="C35" s="10" t="n"/>
@@ -1380,7 +1384,7 @@
       <c r="K35" s="10" t="n"/>
       <c r="L35" s="5" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="27" customHeight="1">
       <c r="A36" s="5" t="n"/>
       <c r="B36" s="5" t="n"/>
       <c r="C36" s="10" t="n"/>
@@ -1394,7 +1398,7 @@
       <c r="K36" s="10" t="n"/>
       <c r="L36" s="5" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="27" customHeight="1">
       <c r="A37" s="5" t="n"/>
       <c r="B37" s="5" t="n"/>
       <c r="C37" s="10" t="n"/>
@@ -1408,7 +1412,7 @@
       <c r="K37" s="10" t="n"/>
       <c r="L37" s="5" t="n"/>
     </row>
-    <row r="38">
+    <row r="38" ht="27" customHeight="1">
       <c r="A38" s="5" t="n"/>
       <c r="B38" s="5" t="n"/>
       <c r="C38" s="10" t="n"/>
@@ -1422,7 +1426,7 @@
       <c r="K38" s="10" t="n"/>
       <c r="L38" s="5" t="n"/>
     </row>
-    <row r="39">
+    <row r="39" ht="27" customHeight="1">
       <c r="A39" s="5" t="n"/>
       <c r="B39" s="5" t="n"/>
       <c r="C39" s="10" t="n"/>
@@ -1436,7 +1440,7 @@
       <c r="K39" s="10" t="n"/>
       <c r="L39" s="5" t="n"/>
     </row>
-    <row r="40">
+    <row r="40" ht="27" customHeight="1">
       <c r="A40" s="5" t="n"/>
       <c r="B40" s="5" t="n"/>
       <c r="C40" s="10" t="n"/>
@@ -1450,7 +1454,7 @@
       <c r="K40" s="10" t="n"/>
       <c r="L40" s="5" t="n"/>
     </row>
-    <row r="41">
+    <row r="41" ht="27" customHeight="1">
       <c r="A41" s="5" t="n"/>
       <c r="B41" s="5" t="n"/>
       <c r="C41" s="10" t="n"/>
@@ -1464,7 +1468,7 @@
       <c r="K41" s="10" t="n"/>
       <c r="L41" s="5" t="n"/>
     </row>
-    <row r="42">
+    <row r="42" ht="27" customHeight="1">
       <c r="A42" s="5" t="n"/>
       <c r="B42" s="5" t="n"/>
       <c r="C42" s="10" t="n"/>
@@ -1478,7 +1482,7 @@
       <c r="K42" s="10" t="n"/>
       <c r="L42" s="5" t="n"/>
     </row>
-    <row r="43">
+    <row r="43" ht="27" customHeight="1">
       <c r="A43" s="5" t="n"/>
       <c r="B43" s="5" t="n"/>
       <c r="C43" s="10" t="n"/>
@@ -1492,7 +1496,7 @@
       <c r="K43" s="10" t="n"/>
       <c r="L43" s="5" t="n"/>
     </row>
-    <row r="44">
+    <row r="44" ht="27" customHeight="1">
       <c r="A44" s="5" t="n"/>
       <c r="B44" s="5" t="n"/>
       <c r="C44" s="10" t="n"/>
@@ -1506,7 +1510,7 @@
       <c r="K44" s="10" t="n"/>
       <c r="L44" s="5" t="n"/>
     </row>
-    <row r="45">
+    <row r="45" ht="27" customHeight="1">
       <c r="A45" s="5" t="n"/>
       <c r="B45" s="5" t="n"/>
       <c r="C45" s="10" t="n"/>
@@ -1520,7 +1524,7 @@
       <c r="K45" s="10" t="n"/>
       <c r="L45" s="5" t="n"/>
     </row>
-    <row r="46">
+    <row r="46" ht="27" customHeight="1">
       <c r="A46" s="5" t="n"/>
       <c r="B46" s="5" t="n"/>
       <c r="C46" s="10" t="n"/>
@@ -1534,7 +1538,7 @@
       <c r="K46" s="10" t="n"/>
       <c r="L46" s="5" t="n"/>
     </row>
-    <row r="47">
+    <row r="47" ht="27" customHeight="1">
       <c r="A47" s="5" t="n"/>
       <c r="B47" s="5" t="n"/>
       <c r="C47" s="10" t="n"/>
@@ -1548,7 +1552,7 @@
       <c r="K47" s="10" t="n"/>
       <c r="L47" s="5" t="n"/>
     </row>
-    <row r="48">
+    <row r="48" ht="27" customHeight="1">
       <c r="A48" s="5" t="n"/>
       <c r="B48" s="5" t="n"/>
       <c r="C48" s="10" t="n"/>
@@ -1562,7 +1566,7 @@
       <c r="K48" s="10" t="n"/>
       <c r="L48" s="5" t="n"/>
     </row>
-    <row r="49">
+    <row r="49" ht="27" customHeight="1">
       <c r="A49" s="5" t="n"/>
       <c r="B49" s="5" t="n"/>
       <c r="C49" s="10" t="n"/>
@@ -1576,7 +1580,7 @@
       <c r="K49" s="10" t="n"/>
       <c r="L49" s="5" t="n"/>
     </row>
-    <row r="50">
+    <row r="50" ht="27" customHeight="1">
       <c r="A50" s="5" t="n"/>
       <c r="B50" s="5" t="n"/>
       <c r="C50" s="10" t="n"/>
@@ -1590,7 +1594,7 @@
       <c r="K50" s="10" t="n"/>
       <c r="L50" s="5" t="n"/>
     </row>
-    <row r="51">
+    <row r="51" ht="27" customHeight="1">
       <c r="A51" s="5" t="n"/>
       <c r="B51" s="5" t="n"/>
       <c r="C51" s="10" t="n"/>
@@ -1604,7 +1608,7 @@
       <c r="K51" s="10" t="n"/>
       <c r="L51" s="5" t="n"/>
     </row>
-    <row r="52">
+    <row r="52" ht="27" customHeight="1">
       <c r="A52" s="5" t="n"/>
       <c r="B52" s="5" t="n"/>
       <c r="C52" s="10" t="n"/>
@@ -1618,7 +1622,7 @@
       <c r="K52" s="10" t="n"/>
       <c r="L52" s="5" t="n"/>
     </row>
-    <row r="53">
+    <row r="53" ht="27" customHeight="1">
       <c r="A53" s="5" t="n"/>
       <c r="B53" s="5" t="n"/>
       <c r="C53" s="10" t="n"/>
@@ -1632,7 +1636,7 @@
       <c r="K53" s="10" t="n"/>
       <c r="L53" s="5" t="n"/>
     </row>
-    <row r="54">
+    <row r="54" ht="27" customHeight="1">
       <c r="A54" s="5" t="n"/>
       <c r="B54" s="5" t="n"/>
       <c r="C54" s="10" t="n"/>
@@ -1731,7 +1735,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="27" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Recuperação Deep Archive BULK</t>
@@ -1755,7 +1759,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
         <f>IF('Dados da transferência'!B11="BULK",IFERROR(B5*D5,"Não precificado"),0)</f>
         <v/>
       </c>
@@ -1770,7 +1774,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="27" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Recuperação Deep Archive STANDARD</t>
@@ -1794,7 +1798,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="13">
         <f>IF('Dados da transferência'!B11="STANDARD",IFERROR(B6*D6,"Não precificado"),0)</f>
         <v/>
       </c>
@@ -1809,7 +1813,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="27" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Cópia temporária restaurada</t>
@@ -1833,7 +1837,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="13">
         <f>IFERROR(B7*D7,"Não precificado")</f>
         <v/>
       </c>
@@ -1848,7 +1852,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="27" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>S3 Batch Operations</t>
@@ -1872,7 +1876,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="13">
         <f>IFERROR(B8*D8,"Não precificado")</f>
         <v/>
       </c>
@@ -1887,7 +1891,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="27" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Tarefas de objeto S3 Batch</t>
@@ -1911,7 +1915,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="13">
         <f>IFERROR(B9*D9,"Não precificado")</f>
         <v/>
       </c>
@@ -1926,7 +1930,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="27" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Discovery e polling de restore</t>
@@ -1950,7 +1954,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="13">
         <f>IFERROR(B10*D10,"Não precificado")</f>
         <v/>
       </c>
@@ -1965,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="27" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Leituras de objetos S3</t>
@@ -1989,7 +1993,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="13">
         <f>IFERROR(B11*D11,"Não precificado")</f>
         <v/>
       </c>
@@ -2004,7 +2008,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="27" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Leituras de tags S3</t>
@@ -2028,7 +2032,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="13">
         <f>IF('Dados da transferência'!B14,IFERROR(B12*D12,"Não precificado"),0)</f>
         <v/>
       </c>
@@ -2043,7 +2047,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="27" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Outbound AWS</t>
@@ -2067,7 +2071,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="13">
         <f>IF(H13,IFERROR(B13*D13,"Não precificado"),0)</f>
         <v/>
       </c>
@@ -2080,7 +2084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="27" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Exclusão antecipada Deep Archive</t>
@@ -2104,7 +2108,7 @@
           <t>AWS pública</t>
         </is>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="13">
         <f>IF('Dados da transferência'!B15&gt;0,IFERROR(B14*D14,"Não precificado"),0)</f>
         <v/>
       </c>
@@ -2119,8 +2123,8 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Custo único por wave</t>
         </is>
@@ -2129,15 +2133,15 @@
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
-      <c r="F16" s="14">
+      <c r="F16" s="15">
         <f>SUM(F5:F13)</f>
         <v/>
       </c>
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Custo único do projeto</t>
         </is>
@@ -2146,7 +2150,7 @@
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
-      <c r="F17" s="14">
+      <c r="F17" s="15">
         <f>F16*'Dados da transferência'!B9+F14</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Use hourly restore retention in cost workbook
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -21,11 +21,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="#,##0.00;[Red]-#,##0.00;—"/>
-    <numFmt numFmtId="165" formatCode="#,##0.;[Red]-#,##0.;—"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00;[Red]-#,##0.00;0"/>
+    <numFmt numFmtId="165" formatCode="#,##0;[Red]-#,##0;0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="$ #,##0.000000;[Red]-$ #,##0.000000;$ 0.000000"/>
-    <numFmt numFmtId="168" formatCode="#,##0.0000;[Red]-#,##0.0000;—"/>
+    <numFmt numFmtId="168" formatCode="#,##0.0000;[Red]-#,##0.0000;0"/>
     <numFmt numFmtId="169" formatCode="$ #,##0.00;[Red]-$ #,##0.00;$ 0.00"/>
   </numFmts>
   <fonts count="7">
@@ -685,15 +685,15 @@
     <row r="12" ht="29" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Retenção do restore (dias)</t>
+          <t>Retenção do restore (horas)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Informe por quantos dias a cópia temporária S3 Standard ficará disponível após o restore terminar. Para Deep Archive BULK, 2 dias é a opção mais segura.</t>
+          <t>Informe por quantas horas a cópia temporária S3 Standard ficará disponível após o restore terminar. Para Deep Archive BULK, 48 horas é a opção mais segura.</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10*'Dados da transferência'!B12/30</f>
+        <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10*'Dados da transferência'!B12/(24*30)</f>
         <v/>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Cópia S3 Standard temporária após o restore.</t>
+          <t>Cópia S3 Standard temporária após o restore; a retenção em horas é convertida para mês.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add total transfer duration estimate to workbook
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -20,13 +20,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.00;[Red]-#,##0.00;0"/>
     <numFmt numFmtId="165" formatCode="#,##0;[Red]-#,##0;0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="$ #,##0.000000;[Red]-$ #,##0.000000;$ 0.000000"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000;[Red]-#,##0.0000;0"/>
     <numFmt numFmtId="169" formatCode="$ #,##0.00;[Red]-$ #,##0.00;$ 0.00"/>
+    <numFmt numFmtId="170" formatCode="[h]&quot; h &quot;mm&quot; min&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -62,7 +63,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +95,11 @@
         <fgColor rgb="000F5132"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00166534"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -166,6 +172,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -533,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -754,6 +763,21 @@
       <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Informe a idade média ponderada desde a entrada no Deep Archive — não use LastModified se a transição foi por lifecycle. Com 180 ou mais, não há cobrança antecipada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="29" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Vazão efetiva estimada (Mbps)</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Informe a vazão média efetiva esperada para a cópia, em Mbps. Use uma taxa sustentável medida ou conservadora — não necessariamente a capacidade nominal do link. É usada somente na estimativa de tempo.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -2157,6 +2181,31 @@
       <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="n"/>
     </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Tempo estimado para transferir todos os dados</t>
+        </is>
+      </c>
+      <c r="B19" s="16">
+        <f>'Dados da transferência'!B6*8000000/'Dados da transferência'!B17/86400</f>
+        <v/>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>duração</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Baseado no volume total e na vazão efetiva configurada. Não inclui restore, filas, pausas, retries ou validações.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
Show transfer duration in months days and hours
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -20,14 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.00;[Red]-#,##0.00;0"/>
     <numFmt numFmtId="165" formatCode="#,##0;[Red]-#,##0;0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="$ #,##0.000000;[Red]-$ #,##0.000000;$ 0.000000"/>
     <numFmt numFmtId="168" formatCode="#,##0.0000;[Red]-#,##0.0000;0"/>
     <numFmt numFmtId="169" formatCode="$ #,##0.00;[Red]-$ #,##0.00;$ 0.00"/>
-    <numFmt numFmtId="170" formatCode="[h]&quot; h &quot;mm&quot; min&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -174,7 +173,7 @@
     <xf numFmtId="169" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2188,12 +2187,12 @@
         </is>
       </c>
       <c r="B19" s="16">
-        <f>'Dados da transferência'!B6*8000000/'Dados da transferência'!B17/86400</f>
+        <f>INT(ROUND('Dados da transferência'!B6*8000000/'Dados da transferência'!B17/3600,0)/(24*30))&amp;" meses, "&amp;INT(MOD(ROUND('Dados da transferência'!B6*8000000/'Dados da transferência'!B17/3600,0),24*30)/24)&amp;" dias e "&amp;MOD(ROUND('Dados da transferência'!B6*8000000/'Dados da transferência'!B17/3600,0),24)&amp;" horas"</f>
         <v/>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>duração</t>
+          <t>meses, dias e horas</t>
         </is>
       </c>
       <c r="D19" s="4" t="n"/>
@@ -2201,7 +2200,7 @@
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Baseado no volume total e na vazão efetiva configurada. Não inclui restore, filas, pausas, retries ou validações.</t>
+          <t>Baseado no volume total e na vazão efetiva configurada. Mês operacional = 30 dias. Não inclui restore, filas, pausas, retries ou validações.</t>
         </is>
       </c>
       <c r="H19" s="4" t="n"/>

</xml_diff>

<commit_message>
Publish optimized Raijin identity and project updates
</commit_message>
<xml_diff>
--- a/docs/raijin-cost-calculator.xlsx
+++ b/docs/raijin-cost-calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\inicoli\TRAMPO\OCI\object_storage\raijin-data-migration_s3-to-oci\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB96B50A-7314-4B17-A58B-1D334855D767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A262CE9-DFDD-4A6D-8A10-8C4C1B4D48AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dados da transferência" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tarifas por região'!$A$4:$L$54</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="87">
   <si>
     <t>RAIJIN — Dados da transferência</t>
   </si>
@@ -138,10 +138,6 @@
   <si>
     <t>Outbound AWS Internet
 US$/GB</t>
-  </si>
-  <si>
-    <t>Armazenamento Deep Archive
-US$/GB-mês</t>
   </si>
   <si>
     <t>Recuperação Deep Archive BULK
@@ -1130,13 +1126,13 @@
     </row>
     <row r="16" spans="1:3" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B16" s="15">
         <v>22</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1174,7 +1170,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:XFC54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
@@ -1232,28 +1228,28 @@
         <v>32</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="22" t="s">
         <v>39</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="K4" s="22" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
@@ -1261,7 +1257,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="21">
         <v>0.15</v>
@@ -1288,15 +1284,15 @@
         <v>1.5E-5</v>
       </c>
       <c r="K5" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="21">
         <v>0.09</v>
@@ -1323,7 +1319,7 @@
         <v>1E-3</v>
       </c>
       <c r="K6" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
@@ -1980,7 +1976,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -1992,7 +1988,7 @@
     </row>
     <row r="2" spans="1:9" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
@@ -2000,7 +1996,7 @@
       <c r="E2" s="36"/>
       <c r="F2" s="36"/>
       <c r="G2" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H2" s="19">
         <v>5.16</v>
@@ -2008,112 +2004,112 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>53</v>
-      </c>
       <c r="H4" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="6">
         <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10</f>
         <v>10000</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D5" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,4,FALSE)</f>
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F5" s="12">
         <f>IF('Dados da transferência'!B11="BULK",IFERROR(B5*D5,"Não precificado"),0)</f>
         <v>80</v>
       </c>
       <c r="G5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" s="6">
         <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10</f>
         <v>10000</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D6" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,5,FALSE)</f>
         <v>2.8000000000000001E-2</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F6" s="12">
         <f>IF('Dados da transferência'!B11="STANDARD",IFERROR(B6*D6,"Não precificado"),0)</f>
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" s="10" t="s">
         <v>57</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" s="6">
         <f>'Dados da transferência'!B8*1000*'Dados da transferência'!B10*'Dados da transferência'!B12/(24*30)</f>
         <v>333.33333333333331</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,6,FALSE)</f>
         <v>4.0500000000000001E-2</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F7" s="12">
-        <f>IF(H7,IFERROR(B7*D7,"Não precificado"),0)</f>
+        <f>IF(H7,IFERROR(B7*D7,"Não precificado"),"-")</f>
         <v>13.5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H7" s="4" t="b">
         <v>1</v>
@@ -2121,28 +2117,28 @@
     </row>
     <row r="8" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B8" s="6">
         <f>1</f>
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D8" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,9,FALSE)</f>
         <v>0.25</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F8" s="12">
-        <f>IF(H8,IFERROR(B8*D8,"Não precificado"),)</f>
+        <f>IF(H8,IFERROR(B8*D8,"Não precificado"),"-")</f>
         <v>0.25</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H8" s="4" t="b">
         <v>1</v>
@@ -2150,28 +2146,28 @@
     </row>
     <row r="9" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B9" s="6">
         <f>ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9,0)</f>
         <v>64000</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D9" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,10,FALSE)</f>
         <v>1.5E-5</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F9" s="12">
-        <f>IF(H9,IFERROR(B9*D9,"Não precificado"),0)</f>
+        <f>IF(H9,IFERROR(B9*D9,"Não precificado"),"-")</f>
         <v>0.96000000000000008</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H9" s="4" t="b">
         <v>1</v>
@@ -2179,28 +2175,28 @@
     </row>
     <row r="10" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B10" s="6">
         <f>(ROUNDUP('Dados da transferência'!B7/1000,0)*'Dados da transferência'!B13)+ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9/1000,0)</f>
         <v>460864</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D10" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,7,FALSE)/1000</f>
         <v>6.9999999999999999E-6</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F10" s="12">
-        <f>IF(H10,IFERROR(B10*D10,"Não precificado"),0)</f>
+        <f>IF(H10,IFERROR(B10*D10,"Não precificado"),"-")</f>
         <v>3.226048</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H10" s="4" t="b">
         <v>1</v>
@@ -2208,28 +2204,28 @@
     </row>
     <row r="11" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" s="6">
         <f>ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9,0)</f>
         <v>64000</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D11" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,8,FALSE)/1000</f>
         <v>5.5999999999999993E-7</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F11" s="12">
-        <f>IF(H11,IFERROR(B11*D11,"Não precificado"),0)</f>
+        <f>IF(H11,IFERROR(B11*D11,"Não precificado"),"-")</f>
         <v>3.5839999999999997E-2</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H11" s="4" t="b">
         <v>1</v>
@@ -2237,57 +2233,57 @@
     </row>
     <row r="12" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B12" s="6">
         <f>ROUNDUP('Dados da transferência'!B7/'Dados da transferência'!B9,0)</f>
         <v>64000</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D12" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,8,FALSE)/1000</f>
         <v>5.5999999999999993E-7</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F12" s="12">
         <f>IF('Dados da transferência'!B14,IFERROR(B12*D12,"Não precificado"),0)</f>
         <v>3.5839999999999997E-2</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B13" s="6">
         <f>'Dados da transferência'!B8*1000</f>
         <v>10000</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" s="11">
         <f>VLOOKUP('Dados da transferência'!B5,'Tarifas por região'!A:K,3,FALSE)</f>
         <v>0.15</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F13" s="12" t="str">
         <f>IF(H13,IFERROR(B13*D13,"Não precificado"),"-")</f>
         <v>-</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H13" s="4" t="b">
         <v>0</v>
@@ -2295,7 +2291,7 @@
     </row>
     <row r="15" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2306,7 +2302,7 @@
         <v>98.007727999999986</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H15" s="17">
         <f>F15*$H$2</f>
@@ -2315,7 +2311,7 @@
     </row>
     <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2334,7 +2330,7 @@
     </row>
     <row r="18" spans="1:8" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B18" s="31" t="str">
         <f>INT(ROUND('Dados da transferência'!B6*8000000/'Dados da transferência'!B15/3600,0)/(24*'Dados da transferência'!B16))&amp;" meses, "&amp;INT(MOD(ROUND('Dados da transferência'!B6*8000000/'Dados da transferência'!B15/3600,0),24*'Dados da transferência'!B16)/24)&amp;" dias e "&amp;MOD(ROUND('Dados da transferência'!B6*8000000/'Dados da transferência'!B15/3600,0),24)&amp;" horas"</f>
@@ -2342,7 +2338,7 @@
       </c>
       <c r="C18" s="32"/>
       <c r="D18" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="33" t="str">
@@ -2371,7 +2367,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="H13 H7:H11" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="H7:H11 H13" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>